<commit_message>
Write the PPFG methodology inside the chart
Adds a methodology panel (steps, calibration, margins, limitations and
references) to the right of the Balad field-generic PPFG plot.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NufppzSsNGBmMyVBwrMssT
</commit_message>
<xml_diff>
--- a/PPFG_Balad/Balad_Unified_PPFG.xlsx
+++ b/PPFG_Balad/Balad_Unified_PPFG.xlsx
@@ -14165,8 +14165,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>45263</xdr:colOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>372694</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>121359</xdr:rowOff>
     </xdr:to>
@@ -14186,7 +14186,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="609600" y="190500"/>
-          <a:ext cx="5531663" cy="6788859"/>
+          <a:ext cx="8297494" cy="6788859"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Add final PPFG chart variant showing the nine offset wells
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NufppzSsNGBmMyVBwrMssT
</commit_message>
<xml_diff>
--- a/PPFG_Balad/Balad_Unified_PPFG.xlsx
+++ b/PPFG_Balad/Balad_Unified_PPFG.xlsx
@@ -19,8 +19,9 @@
     <sheet name="Drilling events" sheetId="10" r:id="rId10"/>
     <sheet name="Chart - Final (approval)" sheetId="11" r:id="rId11"/>
     <sheet name="Chart - QC all wells" sheetId="12" r:id="rId12"/>
-    <sheet name="Chart - OBG QC" sheetId="13" r:id="rId13"/>
-    <sheet name="Method &amp; References" sheetId="14" r:id="rId14"/>
+    <sheet name="Chart - Final with wells" sheetId="13" r:id="rId13"/>
+    <sheet name="Chart - OBG QC" sheetId="14" r:id="rId14"/>
+    <sheet name="Method &amp; References" sheetId="15" r:id="rId15"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -14457,6 +14458,49 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>227976</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>75690</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="Balad_PPFG_Final_Wells.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="190500"/>
+          <a:ext cx="7543176" cy="6171690"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>304581</xdr:colOff>
       <xdr:row>24</xdr:row>
@@ -38675,6 +38719,16 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>

</xml_diff>